<commit_message>
feat: add button create patient for role reception
</commit_message>
<xml_diff>
--- a/map_socket.xlsx
+++ b/map_socket.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8520"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
     <t>Nơi Lắng Nghe &amp; Xử lý (Frontend Listeners)</t>
   </si>
   <si>
-    <t>Bệnh nhân đặt lịch khám thành công</t>
+    <t>Bệnh nhân đặt lịch khám thành công, hoặc lễ tân tạo lịch</t>
   </si>
   <si>
     <t>- Component tab hóa đơn &amp; lịch hẹn trang admin</t>
@@ -759,7 +759,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -771,6 +771,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1057,6 +1066,53 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3651885</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>72390</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4160520"/>
+          <a:ext cx="9267825" cy="5010150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1313,7 +1369,7 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="37.8888888888889" customWidth="1"/>
+    <col min="2" max="2" width="53.8888888888889" customWidth="1"/>
     <col min="3" max="3" width="56.4444444444444" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1333,163 +1389,159 @@
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="4"/>
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="2"/>
+      <c r="A5" s="5"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="2"/>
+      <c r="A6" s="5"/>
       <c r="B6" s="2"/>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="2"/>
+      <c r="A7" s="5"/>
       <c r="B7" s="2"/>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="2"/>
+      <c r="A8" s="5"/>
       <c r="B8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="2"/>
+      <c r="A9" s="5"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="2"/>
+      <c r="A10" s="5"/>
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="2"/>
+      <c r="A11" s="5"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="2"/>
+      <c r="A12" s="5"/>
       <c r="B12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="2"/>
+      <c r="A13" s="5"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="2"/>
+      <c r="A14" s="5"/>
       <c r="B14" s="2"/>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="10" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="2"/>
+      <c r="A15" s="5"/>
       <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="10" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="2"/>
+      <c r="A16" s="6"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="10" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="7"/>
+      <c r="B17" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="10" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="7" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="7" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="7" t="s">
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="7" t="s">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="10" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="10">
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A4:A16"/>
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B4:B7"/>
@@ -1501,5 +1553,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update(websocket): fix bug websocket
</commit_message>
<xml_diff>
--- a/map_socket.xlsx
+++ b/map_socket.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Tên socket</t>
   </si>
@@ -38,6 +38,9 @@
     <t>Nơi Lắng Nghe &amp; Xử lý (Frontend Listeners)</t>
   </si>
   <si>
+    <t>create_appooiment</t>
+  </si>
+  <si>
     <t>Bệnh nhân đặt lịch khám thành công, hoặc lễ tân tạo lịch</t>
   </si>
   <si>
@@ -50,7 +53,7 @@
     <t>update_appoiments</t>
   </si>
   <si>
-    <t>Lễ tân checkin, bác sĩ đổi status(mời, pass, khám xong)</t>
+    <t>Lễ tân checkin, bác sĩ đổi status(mời, pass)</t>
   </si>
   <si>
     <t>- Component MyAppoiment(KH)</t>
@@ -66,6 +69,24 @@
   </si>
   <si>
     <t>- Component BillingManager(LT)</t>
+  </si>
+  <si>
+    <t>invoice_created</t>
+  </si>
+  <si>
+    <t>Khi Bác sĩ khám xong và ấn "Hoàn tất" (Trạng thái ca khám chuyển thành DONE)</t>
+  </si>
+  <si>
+    <t>invoice_paid</t>
+  </si>
+  <si>
+    <t>Hàm update - khi Thu ngân bấm xác nhận thu tiền mặt và đẩy status thành PAID</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Component BillingManager(LT)</t>
+  </si>
+  <si>
+    <t>- Component AdminTransactions(ADMIN)</t>
   </si>
   <si>
     <t xml:space="preserve">Thanh toán thành công </t>
@@ -490,19 +511,6 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -518,6 +526,19 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -768,7 +789,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -781,31 +802,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
@@ -1097,7 +1121,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3651885</xdr:colOff>
+      <xdr:colOff>2882265</xdr:colOff>
       <xdr:row>49</xdr:row>
       <xdr:rowOff>72390</xdr:rowOff>
     </xdr:to>
@@ -1387,7 +1411,7 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="53.8888888888889" customWidth="1"/>
+    <col min="2" max="2" width="65.1111111111111" customWidth="1"/>
     <col min="3" max="3" width="56.4444444444444" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1403,79 +1427,95 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:3">
-      <c r="A2" s="2"/>
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="13" t="s">
         <v>4</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="13" t="s">
-        <v>5</v>
+      <c r="C3" s="14" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="13" t="s">
         <v>8</v>
       </c>
+      <c r="C4" s="14" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="13" t="s">
-        <v>9</v>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="14" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="13" t="s">
-        <v>10</v>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="14" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="13" t="s">
-        <v>11</v>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="14" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="13" t="s">
-        <v>12</v>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="14" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="3"/>
+      <c r="A9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="3"/>
+      <c r="A10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="3"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="14" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
-      <c r="C12" s="3"/>
+      <c r="C12" s="7"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="6"/>
@@ -1484,69 +1524,71 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="6"/>
-      <c r="B14" s="7"/>
+      <c r="B14" s="8"/>
       <c r="C14" s="3"/>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="8"/>
+      <c r="A15" s="9"/>
       <c r="B15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>14</v>
+        <v>20</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="9"/>
+      <c r="A16" s="10"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="13" t="s">
-        <v>15</v>
+      <c r="C16" s="14" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>17</v>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="13" t="s">
-        <v>18</v>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="14" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="13" t="s">
-        <v>19</v>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="14" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="13" t="s">
-        <v>20</v>
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="14" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13" t="s">
-        <v>21</v>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="14" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A9"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="A10:A11"/>
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B9"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="B17:B21"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat(AI suggest): basic API Gemini
</commit_message>
<xml_diff>
--- a/map_socket.xlsx
+++ b/map_socket.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Tên socket</t>
   </si>
@@ -38,19 +38,16 @@
     <t>Nơi Lắng Nghe &amp; Xử lý (Frontend Listeners)</t>
   </si>
   <si>
-    <t>create_appooiment</t>
+    <t>appointment_created</t>
   </si>
   <si>
     <t>Bệnh nhân đặt lịch khám thành công, hoặc lễ tân tạo lịch</t>
   </si>
   <si>
-    <t>- Component tab hóa đơn &amp; lịch hẹn trang admin</t>
-  </si>
-  <si>
-    <t>- Component tab lịch hẹn trang lễ tân</t>
-  </si>
-  <si>
-    <t>update_appoiments</t>
+    <t>- Component AppointmentMonitor(LT)</t>
+  </si>
+  <si>
+    <t>appointment_updated</t>
   </si>
   <si>
     <t>Lễ tân checkin, bác sĩ đổi status(mời, pass)</t>
@@ -62,21 +59,21 @@
     <t>- Component ClinicQueue(LT)</t>
   </si>
   <si>
-    <t>- Component AppointmentMonitor(LT)</t>
-  </si>
-  <si>
-    <t>- Component DoctorClinicQueue(BS)</t>
+    <t xml:space="preserve">- Component AppointmentMonitor(LT) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Component DoctorClinicQueue(BS) </t>
+  </si>
+  <si>
+    <t>invoice_created</t>
+  </si>
+  <si>
+    <t>Khi Bác sĩ khám xong và ấn "Hoàn tất" (Trạng thái ca khám chuyển thành DONE)</t>
   </si>
   <si>
     <t>- Component BillingManager(LT)</t>
   </si>
   <si>
-    <t>invoice_created</t>
-  </si>
-  <si>
-    <t>Khi Bác sĩ khám xong và ấn "Hoàn tất" (Trạng thái ca khám chuyển thành DONE)</t>
-  </si>
-  <si>
     <t>invoice_paid</t>
   </si>
   <si>
@@ -87,33 +84,6 @@
   </si>
   <si>
     <t>- Component AdminTransactions(ADMIN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thanh toán thành công </t>
-  </si>
-  <si>
-    <t>- Component hóa đơn &amp; lịch hẹn trang admin</t>
-  </si>
-  <si>
-    <t>- Mấy componnent bên dashboard khách hàng</t>
-  </si>
-  <si>
-    <t>Khách hàng, lễ tân, admin hủy lịch</t>
-  </si>
-  <si>
-    <t>- Component lịch hẹn lễ tân</t>
-  </si>
-  <si>
-    <t>- Component hàng đợi trang bác sĩ</t>
-  </si>
-  <si>
-    <t>- Component hàng đợi phòng khám trang lễ tân</t>
-  </si>
-  <si>
-    <t>- Component ở lịch hẹn của tôi trang dashboard khách hàng</t>
-  </si>
-  <si>
-    <t>- Component tab hóa đơn &amp; lịch hẹn, thống kê tổng quan trang admin</t>
   </si>
 </sst>
 </file>
@@ -481,7 +451,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -502,43 +472,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -665,7 +598,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -677,34 +610,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -789,51 +722,36 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1108,53 +1026,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2882265</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>72390</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="4160520"/>
-          <a:ext cx="9267825" cy="5010150"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1433,83 +1304,79 @@
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="14" t="s">
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="14" t="s">
+    <row r="6" spans="1:3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="14" t="s">
+    <row r="7" spans="1:3">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="14" t="s">
+    <row r="8" spans="1:3">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="14" t="s">
+      <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="4" t="s">
+      <c r="C9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="5" t="s">
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="14" t="s">
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="9" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="14" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1520,80 +1387,59 @@
     <row r="13" spans="1:3">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
-      <c r="C13" s="3"/>
+      <c r="C13" s="7"/>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="6"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="3"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>21</v>
-      </c>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="14" t="s">
-        <v>22</v>
-      </c>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7"/>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>24</v>
-      </c>
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7"/>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="14" t="s">
-        <v>25</v>
-      </c>
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7"/>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="14" t="s">
-        <v>26</v>
-      </c>
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="7"/>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="14" t="s">
-        <v>27</v>
-      </c>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7"/>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="14" t="s">
-        <v>28</v>
-      </c>
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="7">
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="A4:A7"/>
     <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A17:A21"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="B4:B7"/>
     <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B17:B21"/>
+    <mergeCell ref="C2:C3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>